<commit_message>
feat(vehicle_setting): resolve branch-3 rows and regenerate the vf230 revise draft
Run the second-pass lookup over the 105 branch-3 rows: 54 resolve through the
No.267 AUX switch family gate, 3 through a quoted-form FIP condition the v3
parser could not read, 16 turn out to sit on a constant FIP row that needs no
PROXI at all, and 32 stay PENDING. That drops PROXI_PENDING from 105 to 32.

Regenerate the vf230 sandbox draft against the v4 report, keeping the v3 draft
as a backup, and add a fourth data-request section for the 32 remaining rows,
which are settings whose name resolves but whose display condition no source
records.
</commit_message>
<xml_diff>
--- a/features/vehicle_setting/sandbox/vssl/vf230_vssl.xlsx
+++ b/features/vehicle_setting/sandbox/vssl/vf230_vssl.xlsx
@@ -4680,7 +4680,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Power Mode" customer setting is set to BATTERY
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K12" s="78" t="inlineStr">
@@ -4782,7 +4782,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Power Mode" customer setting is set to IGNITION
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K13" s="78" t="inlineStr">
@@ -4884,7 +4884,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K14" s="78" t="inlineStr">
@@ -4993,7 +4993,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Power Mode" customer setting is set to BATTERY
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K15" s="78" t="inlineStr">
@@ -5095,7 +5095,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Power Mode" customer setting is set to IGNITION
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K16" s="78" t="inlineStr">
@@ -5197,7 +5197,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K17" s="78" t="inlineStr">
@@ -5306,7 +5306,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K18" s="78" t="inlineStr">
@@ -5408,7 +5408,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K19" s="78" t="inlineStr">
@@ -5510,7 +5510,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K20" s="78" t="inlineStr">
@@ -5612,7 +5612,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K21" s="78" t="inlineStr">
@@ -5721,7 +5721,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K22" s="78" t="inlineStr">
@@ -5823,7 +5823,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K23" s="78" t="inlineStr">
@@ -5925,7 +5925,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K24" s="78" t="inlineStr">
@@ -6034,7 +6034,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K25" s="78" t="inlineStr">
@@ -6136,7 +6136,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 5 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K26" s="78" t="inlineStr">
@@ -6238,7 +6238,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K27" s="78" t="inlineStr">
@@ -6347,7 +6347,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K28" s="78" t="inlineStr">
@@ -6449,7 +6449,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 6 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K29" s="78" t="inlineStr">
@@ -6551,7 +6551,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K30" s="78" t="inlineStr">
@@ -7338,8 +7338,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Rear Guidance Light Status" customer setting is set to ON
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Rear Guidance Light Status" customer setting is set to ON</t>
         </is>
       </c>
       <c r="K38" s="78" t="inlineStr">
@@ -7436,8 +7435,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Rear Guidance Light Status" customer setting is set to OFF
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Rear Guidance Light Status" customer setting is set to OFF</t>
         </is>
       </c>
       <c r="K39" s="78" t="inlineStr">
@@ -7534,8 +7532,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The Vehicle Settings menu is open</t>
         </is>
       </c>
       <c r="K40" s="78" t="inlineStr">
@@ -12885,8 +12882,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Phone Repetition" customer setting is set to On
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Phone Repetition" customer setting is set to On</t>
         </is>
       </c>
       <c r="K94" s="78" t="inlineStr">
@@ -12987,8 +12983,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Phone Repetition" customer setting is set to Off
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Phone Repetition" customer setting is set to Off</t>
         </is>
       </c>
       <c r="K95" s="78" t="inlineStr">
@@ -13089,8 +13084,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The Vehicle Settings menu is open</t>
         </is>
       </c>
       <c r="K96" s="78" t="inlineStr">
@@ -18961,8 +18955,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The Vehicle Settings menu is open</t>
         </is>
       </c>
       <c r="K155" s="87" t="inlineStr">
@@ -27672,7 +27665,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K243" s="78" t="inlineStr">
@@ -27774,7 +27767,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K244" s="78" t="inlineStr">
@@ -27883,7 +27876,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K245" s="78" t="inlineStr">
@@ -27985,7 +27978,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K246" s="78" t="inlineStr">
@@ -28087,7 +28080,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K247" s="78" t="inlineStr">
@@ -28196,7 +28189,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K248" s="78" t="inlineStr">
@@ -28298,7 +28291,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K249" s="78" t="inlineStr">
@@ -28400,7 +28393,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K250" s="78" t="inlineStr">
@@ -28509,7 +28502,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Type" customer setting is set to Momentary
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K251" s="78" t="inlineStr">
@@ -28611,7 +28604,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Type" customer setting is set to Latching
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K252" s="78" t="inlineStr">
@@ -28713,7 +28706,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K253" s="78" t="inlineStr">
@@ -28822,7 +28815,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K254" s="78" t="inlineStr">
@@ -28924,7 +28917,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K255" s="78" t="inlineStr">
@@ -29026,7 +29019,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K256" s="78" t="inlineStr">
@@ -29135,7 +29128,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K257" s="78" t="inlineStr">
@@ -29237,7 +29230,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K258" s="78" t="inlineStr">
@@ -29339,7 +29332,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K259" s="78" t="inlineStr">
@@ -29448,7 +29441,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K260" s="78" t="inlineStr">
@@ -29550,7 +29543,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K261" s="78" t="inlineStr">
@@ -29652,7 +29645,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K262" s="78" t="inlineStr">
@@ -29761,7 +29754,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Hold Last State" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K263" s="78" t="inlineStr">
@@ -29863,7 +29856,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Hold Last State" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K264" s="78" t="inlineStr">
@@ -29965,7 +29958,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K265" s="78" t="inlineStr">
@@ -31781,8 +31774,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Suspension Default Ride Height" customer setting is set to Aerodynamic
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Suspension Default Ride Height" customer setting is set to Aerodynamic</t>
         </is>
       </c>
       <c r="K283" s="78" t="inlineStr">
@@ -31881,8 +31873,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Suspension Default Ride Height" customer setting is set to Normal
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Suspension Default Ride Height" customer setting is set to Normal</t>
         </is>
       </c>
       <c r="K284" s="78" t="inlineStr">
@@ -31981,8 +31972,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The Vehicle Settings menu is open</t>
         </is>
       </c>
       <c r="K285" s="78" t="inlineStr">
@@ -32187,7 +32177,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Power Mode" customer setting is set to Battery
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K287" s="78" t="inlineStr">
@@ -32289,7 +32279,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 1 Power Mode" customer setting is set to Ignition
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K288" s="78" t="inlineStr">
@@ -32391,7 +32381,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K289" s="78" t="inlineStr">
@@ -32500,7 +32490,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Power Mode" customer setting is set to Battery
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K290" s="78" t="inlineStr">
@@ -32602,7 +32592,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 2 Power Mode" customer setting is set to Ignition
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K291" s="78" t="inlineStr">
@@ -32704,7 +32694,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K292" s="78" t="inlineStr">
@@ -32813,7 +32803,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Power Mode" customer setting is set to Battery
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K293" s="78" t="inlineStr">
@@ -32915,7 +32905,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 3 Power Mode" customer setting is set to Ignition
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K294" s="87" t="inlineStr">
@@ -33017,7 +33007,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K295" s="87" t="inlineStr">
@@ -33126,7 +33116,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Power Mode" customer setting is set to Battery
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K296" s="87" t="inlineStr">
@@ -33228,7 +33218,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "SWITCH 4 Power Mode" customer setting is set to Ignition
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K297" s="87" t="inlineStr">
@@ -33330,7 +33320,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K298" s="87" t="inlineStr">
@@ -35604,8 +35594,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Ready to Drive Pop-Up" customer setting is set to On
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Ready to Drive Pop-Up" customer setting is set to On</t>
         </is>
       </c>
       <c r="K321" s="87" t="inlineStr">
@@ -35704,8 +35693,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The "Ready to Drive Pop-Up" customer setting is set to Off
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The "Ready to Drive Pop-Up" customer setting is set to Off</t>
         </is>
       </c>
       <c r="K322" s="87" t="inlineStr">
@@ -35804,8 +35792,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. The Vehicle Settings menu is open</t>
         </is>
       </c>
       <c r="K323" s="87" t="inlineStr">
@@ -36101,7 +36088,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Auto Fold Mirrors" customer setting is set to On
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Auto_Power_Folding_Mirrors = 1 (Present)</t>
         </is>
       </c>
       <c r="K326" s="87" t="inlineStr">
@@ -36199,7 +36186,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Auto Fold Mirrors" customer setting is set to Off
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Auto_Power_Folding_Mirrors = 1 (Present)</t>
         </is>
       </c>
       <c r="K327" s="87" t="inlineStr">
@@ -36297,7 +36284,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Auto_Power_Folding_Mirrors = 1 (Present)</t>
         </is>
       </c>
       <c r="K328" s="87" t="inlineStr">
@@ -46334,8 +46321,7 @@
       </c>
       <c r="J428" s="95" t="inlineStr">
         <is>
-          <t>1. The HU is in the Full-Operation state
-2. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+          <t>1. The HU is in the Full-Operation state</t>
         </is>
       </c>
       <c r="K428" s="78" t="inlineStr">
@@ -46432,8 +46418,7 @@
       </c>
       <c r="J429" s="95" t="inlineStr">
         <is>
-          <t>1. The HU is in the Full-Operation state
-2. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+          <t>1. The HU is in the Full-Operation state</t>
         </is>
       </c>
       <c r="K429" s="78" t="inlineStr">
@@ -46530,8 +46515,7 @@
       </c>
       <c r="J430" s="95" t="inlineStr">
         <is>
-          <t>1. The HU is in the Full-Operation state
-2. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+          <t>1. The HU is in the Full-Operation state</t>
         </is>
       </c>
       <c r="K430" s="78" t="inlineStr">

</xml_diff>

<commit_message>
fix(vehicle_setting): drop contradictory preconditions and resolve negated conditions
Remove the 'menu is open' precondition from the 52 rows whose procedure now
builds that state itself through the inserted navigation steps, leaving the 38
rows without navigation untouched. Resolve the two negated FIP conditions with
a representative value from the spec value table, which drops PROXI_PENDING
from 32 to 25 and shrinks the fourth data-request section to 9 names.
Correct an inherited FO section citation that belongs to IN.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GKkNpeyaVaKVBYBPWdfuXU
</commit_message>
<xml_diff>
--- a/features/vehicle_setting/sandbox/vssl/vf230_vssl.xlsx
+++ b/features/vehicle_setting/sandbox/vssl/vf230_vssl.xlsx
@@ -4883,8 +4883,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K14" s="78" t="inlineStr">
@@ -5196,8 +5195,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K17" s="78" t="inlineStr">
@@ -5611,8 +5609,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K21" s="78" t="inlineStr">
@@ -5924,8 +5921,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K24" s="78" t="inlineStr">
@@ -6237,8 +6233,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K27" s="78" t="inlineStr">
@@ -6550,8 +6545,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 2 (Type 2)</t>
+3. PROXI AUX_Switch_Types = 2 (Type 2)</t>
         </is>
       </c>
       <c r="K30" s="78" t="inlineStr">
@@ -8321,8 +8315,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Blind_Spot_Monitoring = 1 (Present)</t>
+3. PROXI Blind_Spot_Monitoring = 1 (Present)</t>
         </is>
       </c>
       <c r="K48" s="78" t="inlineStr">
@@ -8821,8 +8814,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Passive_Entry_Menu = 1 (Present)</t>
+3. PROXI Passive_Entry_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K53" s="78" t="inlineStr">
@@ -9809,8 +9801,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Auto_Park_Brake_Menu = 1 (Present)</t>
+3. PROXI Auto_Park_Brake_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K63" s="78" t="inlineStr">
@@ -11383,8 +11374,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Auto_Door_Unlock_Menu = 1 (Present)</t>
+3. PROXI Auto_Door_Unlock_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K79" s="78" t="inlineStr">
@@ -12371,8 +12361,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K89" s="78" t="inlineStr">
@@ -12573,8 +12562,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K91" s="78" t="inlineStr">
@@ -13083,8 +13071,7 @@
       <c r="J96" s="95" t="inlineStr">
         <is>
           <t>1. The HU is in the Full-Operation state
-2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open</t>
+2. FD-CAN8 is connected to the bus simulator with signal tracing enabled</t>
         </is>
       </c>
       <c r="K96" s="78" t="inlineStr">
@@ -13487,8 +13474,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K100" s="87" t="inlineStr">
@@ -13894,8 +13880,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K104" s="78" t="inlineStr">
@@ -15484,11 +15469,10 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Heated_Seats = 0 (Absent)
-5. PROXI Else If Heated_Seats = ? (Front Seats)
-6. PROXI Remote_Start = 0 (Absent)
-7. PROXI Else If Remote_Start = ? (Present)</t>
+3. PROXI Heated_Seats = 0 (Absent)
+4. PROXI Else If Heated_Seats = ? (Front Seats)
+5. PROXI Remote_Start = 0 (Absent)
+6. PROXI Else If Remote_Start = ? (Present)</t>
         </is>
       </c>
       <c r="K120" s="78" t="inlineStr">
@@ -15893,11 +15877,10 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Heated_Seats = 0 (Absent)
-5. PROXI Else If Heated_Seats = ? (Front Seats)
-6. PROXI Remote_Start = 0 (Absent)
-7. PROXI Else If Remote_Start = ? (Present)</t>
+3. PROXI Heated_Seats = 0 (Absent)
+4. PROXI Else If Heated_Seats = ? (Front Seats)
+5. PROXI Remote_Start = 0 (Absent)
+6. PROXI Else If Remote_Start = ? (Present)</t>
         </is>
       </c>
       <c r="K124" s="78" t="inlineStr">
@@ -17169,8 +17152,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Cornering_Light = 1 (Present)</t>
+3. PROXI Cornering_Light = 1 (Present)</t>
         </is>
       </c>
       <c r="K137" s="78" t="inlineStr">
@@ -17469,8 +17451,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Greeting_Lights_Menu = 1 (Present)</t>
+3. PROXI Greeting_Lights_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K140" s="87" t="inlineStr">
@@ -18061,8 +18042,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K146" s="87" t="inlineStr">
@@ -18657,8 +18637,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Forward_Collision_Mitigation = 3 (Full Speed Forward Collision Warning with Mitigation)</t>
+3. PROXI Forward_Collision_Mitigation = 3 (Full Speed Forward Collision Warning with Mitigation)</t>
         </is>
       </c>
       <c r="K152" s="78" t="inlineStr">
@@ -19254,8 +19233,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Forward_Collision_Mitigation = 2 (Full Speed FCW with Pedestrian Emergency Braking)</t>
+3. PROXI Forward_Collision_Mitigation = 2 (Full Speed FCW with Pedestrian Emergency Braking)</t>
         </is>
       </c>
       <c r="K158" s="78" t="inlineStr">
@@ -19556,8 +19534,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Rain_Sensor = 1 (Present)</t>
+3. PROXI Rain_Sensor = 1 (Present)</t>
         </is>
       </c>
       <c r="K161" s="78" t="inlineStr">
@@ -19956,8 +19933,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Enable = ? (Enable)</t>
+3. PROXI Enable = ? (Enable)</t>
         </is>
       </c>
       <c r="K165" s="78" t="inlineStr">
@@ -20058,8 +20034,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Enable = ? (Enable)</t>
+3. PROXI Enable = ? (Enable)</t>
         </is>
       </c>
       <c r="K166" s="78" t="inlineStr">
@@ -21548,8 +21523,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Tyre_Pressure_Unit_Menu = 1 (Present)</t>
+3. PROXI Tyre_Pressure_Unit_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K181" s="78" t="inlineStr">
@@ -24296,8 +24270,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI CAN node 82 (PTGM) = 1 (Present)</t>
+3. PROXI CAN node 82 (PTGM) = 1 (Present)</t>
         </is>
       </c>
       <c r="K209" s="78" t="inlineStr">
@@ -24695,8 +24668,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI CAN node 82 (PTGM) = 1 (Present)</t>
+3. PROXI CAN node 82 (PTGM) = 1 (Present)</t>
         </is>
       </c>
       <c r="K213" s="78" t="inlineStr">
@@ -25394,8 +25366,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Traffic_Sign_Recognition_Menu = 1 (Present)</t>
+3. PROXI Traffic_Sign_Recognition_Menu = 1 (Present)</t>
         </is>
       </c>
       <c r="K220" s="78" t="inlineStr">
@@ -25994,8 +25965,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K226" s="87" t="inlineStr">
@@ -26778,8 +26748,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI FOA _Presence = 1 (Present)</t>
+3. PROXI FOA _Presence = 1 (Present)</t>
         </is>
       </c>
       <c r="K234" s="87" t="inlineStr">
@@ -27766,8 +27735,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K244" s="78" t="inlineStr">
@@ -28079,8 +28047,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K247" s="78" t="inlineStr">
@@ -28392,8 +28359,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K250" s="78" t="inlineStr">
@@ -28705,8 +28671,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K253" s="78" t="inlineStr">
@@ -29018,8 +28983,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K256" s="78" t="inlineStr">
@@ -29331,8 +29295,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K259" s="78" t="inlineStr">
@@ -29644,8 +29607,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K262" s="78" t="inlineStr">
@@ -29957,8 +29919,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K265" s="78" t="inlineStr">
@@ -31971,8 +31932,7 @@
       <c r="J285" s="95" t="inlineStr">
         <is>
           <t>1. The HU is in the Full-Operation state
-2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open</t>
+2. FD-CAN8 is connected to the bus simulator with signal tracing enabled</t>
         </is>
       </c>
       <c r="K285" s="78" t="inlineStr">
@@ -32380,8 +32340,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K289" s="78" t="inlineStr">
@@ -32693,8 +32652,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K292" s="78" t="inlineStr">
@@ -33006,8 +32964,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K295" s="87" t="inlineStr">
@@ -33319,8 +33276,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI AUX_Switch_Types = 1 (Type 1)</t>
+3. PROXI AUX_Switch_Types = 1 (Type 1)</t>
         </is>
       </c>
       <c r="K298" s="87" t="inlineStr">
@@ -33830,8 +33786,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+3. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
         </is>
       </c>
       <c r="K303" s="78" t="inlineStr">
@@ -35791,8 +35746,7 @@
       <c r="J323" s="87" t="inlineStr">
         <is>
           <t>1. The HU is in the Full-Operation state
-2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open</t>
+2. FD-CAN8 is connected to the bus simulator with signal tracing enabled</t>
         </is>
       </c>
       <c r="K323" s="87" t="inlineStr">
@@ -36870,7 +36824,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Engine Off Power Delay" customer setting is set to Fourty_Five_Sec
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Country_Code = 2 (United States of America)</t>
         </is>
       </c>
       <c r="K334" s="87" t="inlineStr">
@@ -36968,7 +36922,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Engine Off Power Delay" customer setting is set to Zero
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Country_Code = 2 (United States of America)</t>
         </is>
       </c>
       <c r="K335" s="78" t="inlineStr">
@@ -37066,7 +37020,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Engine Off Power Delay" customer setting is set to Zero
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Country_Code = 2 (United States of America)</t>
         </is>
       </c>
       <c r="K336" s="78" t="inlineStr">
@@ -37164,7 +37118,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Country_Code = 2 (United States of America)</t>
         </is>
       </c>
       <c r="K337" s="78" t="inlineStr">
@@ -37659,8 +37613,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Presence = ? (Present)</t>
+3. PROXI Presence = ? (Present)</t>
         </is>
       </c>
       <c r="K342" s="78" t="inlineStr">
@@ -38159,8 +38112,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI Twilight_Sensor = 1 (Present)</t>
+3. PROXI Twilight_Sensor = 1 (Present)</t>
         </is>
       </c>
       <c r="K347" s="78" t="inlineStr">
@@ -38463,8 +38415,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI CAN node 95 (ITBM/ITCM) = 1 (Present)</t>
+3. PROXI CAN node 95 (ITBM/ITCM) = 1 (Present)</t>
         </is>
       </c>
       <c r="K350" s="78" t="inlineStr">
@@ -39064,7 +39015,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Automatic Trailer Light Check" customer setting is set to Enable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Trailer_Light_Check = 1 (Type 1 (Radio))</t>
         </is>
       </c>
       <c r="K356" s="78" t="inlineStr">
@@ -39162,7 +39113,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The "Automatic Trailer Light Check" customer setting is set to Disable
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Trailer_Light_Check = 1 (Type 1 (Radio))</t>
         </is>
       </c>
       <c r="K357" s="78" t="inlineStr">
@@ -39260,7 +39211,7 @@
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
 3. The Vehicle Settings menu is open
-4. PENDING: DR（未取號，依審閱 §2.2：未送出前不佔號）</t>
+4. PROXI Trailer_Light_Check = 1 (Type 1 (Radio))</t>
         </is>
       </c>
       <c r="K358" s="78" t="inlineStr">
@@ -40273,8 +40224,7 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI CAN node 97 (PSSM) = 1 (Present)</t>
+3. PROXI CAN node 97 (PSSM) = 1 (Present)</t>
         </is>
       </c>
       <c r="K368" s="78" t="inlineStr">
@@ -41699,9 +41649,8 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI (Traffic_Sign_Recognition_Menu = 1 (Present)
-5. PROXI Else If (Traffic_Sign_Recognition_Menu = ? (Present)</t>
+3. PROXI (Traffic_Sign_Recognition_Menu = 1 (Present)
+4. PROXI Else If (Traffic_Sign_Recognition_Menu = ? (Present)</t>
         </is>
       </c>
       <c r="K382" s="78" t="inlineStr">
@@ -43423,9 +43372,8 @@
         <is>
           <t>1. The HU is in the Full-Operation state
 2. FD-CAN8 is connected to the bus simulator with signal tracing enabled
-3. The Vehicle Settings menu is open
-4. PROXI (Traffic_Sign_Recognition_Menu = 1 (Present)
-5. PROXI Else If (Traffic_Sign_Recognition_Menu = ? (Present)</t>
+3. PROXI (Traffic_Sign_Recognition_Menu = 1 (Present)
+4. PROXI Else If (Traffic_Sign_Recognition_Menu = ? (Present)</t>
         </is>
       </c>
       <c r="K399" s="78" t="inlineStr">

</xml_diff>